<commit_message>
feat: tag AY115 demo student names by group (續領/匯入/新申請)
Prefix the demo cohort names so a tester can tell at a glance which
flow a student belongs to: 續領- (114 recipients), 匯入- (批次匯入 workbook),
新申請- (wizard applicants). Applied consistently to the seed, the mock
SIS and the regenerated sample workbooks.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NYWYzgwV9y9wWYJfsQ27SP
</commit_message>
<xml_diff>
--- a/docs/samples/ay115/115_批次匯入.xlsx
+++ b/docs/samples/ay115/115_批次匯入.xlsx
@@ -427,7 +427,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="26" customWidth="1" min="5" max="5"/>
@@ -492,7 +492,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>陳柏宇</t>
+          <t>匯入-陳柏宇</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -535,7 +535,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>李欣怡</t>
+          <t>匯入-李欣怡</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -578,7 +578,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>王志豪</t>
+          <t>匯入-王志豪</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -621,7 +621,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>劉育綺</t>
+          <t>匯入-劉育綺</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">

</xml_diff>